<commit_message>
Prepare portfolio for deployment with Resend
</commit_message>
<xml_diff>
--- a/visitors.xlsx
+++ b/visitors.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="28.44140625" customWidth="1" min="1" max="1"/>
@@ -503,6 +503,33 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-09-25 03:16:28</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Ihtisham Mujahid</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ihtisham191181@gmail.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>+923488282922</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>testing email</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>